<commit_message>
small fix for 1 task
</commit_message>
<xml_diff>
--- a/phase-1/MAI.xlsx
+++ b/phase-1/MAI.xlsx
@@ -171,6 +171,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0000000000"/>
+    <numFmt numFmtId="165" formatCode="0.000000000"/>
+  </numFmts>
   <fonts count="10">
     <font>
       <sz val="10.0"/>
@@ -434,7 +438,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="68">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -588,8 +592,17 @@
     <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -2863,29 +2876,29 @@
         <v>15</v>
       </c>
       <c r="N51" s="42">
-        <f t="shared" ref="N51:N54" si="27">B51/$B$37</f>
-        <v>0.1376467601</v>
+        <f t="shared" ref="N51:Q51" si="26">B51/B$56</f>
+        <v>0.510563553</v>
       </c>
       <c r="O51" s="42">
-        <f t="shared" ref="O51:O54" si="28">C51/$C$37</f>
-        <v>1.916306699</v>
+        <f t="shared" si="26"/>
+        <v>0.425964256</v>
       </c>
       <c r="P51" s="42">
-        <f t="shared" ref="P51:P54" si="29">D51/$D$37</f>
-        <v>0.404122183</v>
+        <f t="shared" si="26"/>
+        <v>0.5918606209</v>
       </c>
       <c r="Q51" s="42">
-        <f t="shared" ref="Q51:Q54" si="30">E51/$E$37</f>
-        <v>0.2867935955</v>
+        <f t="shared" si="26"/>
+        <v>0.3673554265</v>
       </c>
       <c r="R51" s="3"/>
       <c r="S51" s="3">
-        <f t="shared" ref="S51:S54" si="31">AVERAGE(N51:R51)</f>
-        <v>0.6862173094</v>
+        <f t="shared" ref="S51:S54" si="29">AVERAGE(N51:R51)</f>
+        <v>0.4739359641</v>
       </c>
       <c r="T51" s="20">
-        <f t="shared" ref="T51:T54" si="32">AVERAGE(N51:R51)</f>
-        <v>0.6862173094</v>
+        <f t="shared" ref="T51:T54" si="30">AVERAGE(N51:R51)</f>
+        <v>0.4739359641</v>
       </c>
       <c r="U51" s="3"/>
     </row>
@@ -2894,19 +2907,19 @@
         <v>16</v>
       </c>
       <c r="B52" s="42">
-        <f t="shared" ref="B52:E52" si="26">POWER(B43*H43*O43,1/3)</f>
+        <f t="shared" ref="B52:E52" si="27">POWER(B43*H43*O43,1/3)</f>
         <v>0.3218297949</v>
       </c>
       <c r="C52" s="42">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>1</v>
       </c>
       <c r="D52" s="42">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0.3466806372</v>
       </c>
       <c r="E52" s="42">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>3.301927249</v>
       </c>
       <c r="F52" s="36"/>
@@ -2924,29 +2937,29 @@
         <v>16</v>
       </c>
       <c r="N52" s="42">
-        <f t="shared" si="27"/>
-        <v>0.04429882857</v>
+        <f t="shared" ref="N52:Q52" si="28">B52/B$56</f>
+        <v>0.1643145635</v>
       </c>
       <c r="O52" s="42">
         <f t="shared" si="28"/>
-        <v>0.6167245918</v>
+        <v>0.1370879891</v>
       </c>
       <c r="P52" s="42">
-        <f t="shared" si="29"/>
-        <v>0.06119489507</v>
+        <f t="shared" si="28"/>
+        <v>0.08962351019</v>
       </c>
       <c r="Q52" s="42">
-        <f t="shared" si="30"/>
-        <v>0.1893943176</v>
+        <f t="shared" si="28"/>
+        <v>0.2425961785</v>
       </c>
       <c r="R52" s="3"/>
       <c r="S52" s="3">
-        <f t="shared" si="31"/>
-        <v>0.2279031583</v>
+        <f t="shared" si="29"/>
+        <v>0.1584055603</v>
       </c>
       <c r="T52" s="20">
-        <f t="shared" si="32"/>
-        <v>0.2279031583</v>
+        <f t="shared" si="30"/>
+        <v>0.1584055603</v>
       </c>
       <c r="U52" s="3"/>
     </row>
@@ -2955,19 +2968,19 @@
         <v>17</v>
       </c>
       <c r="B53" s="42">
-        <f t="shared" ref="B53:E53" si="33">POWER(B44*H44*O44,1/3)</f>
+        <f t="shared" ref="B53:E53" si="31">POWER(B44*H44*O44,1/3)</f>
         <v>0.4367902324</v>
       </c>
       <c r="C53" s="42">
-        <f t="shared" si="33"/>
+        <f t="shared" si="31"/>
         <v>2.884499141</v>
       </c>
       <c r="D53" s="42">
-        <f t="shared" si="33"/>
+        <f t="shared" si="31"/>
         <v>1</v>
       </c>
       <c r="E53" s="42">
-        <f t="shared" si="33"/>
+        <f t="shared" si="31"/>
         <v>4.30886938</v>
       </c>
       <c r="F53" s="36"/>
@@ -2985,29 +2998,29 @@
         <v>17</v>
       </c>
       <c r="N53" s="42">
-        <f t="shared" si="27"/>
-        <v>0.06012276034</v>
+        <f t="shared" ref="N53:Q53" si="32">B53/B$56</f>
+        <v>0.2230091729</v>
       </c>
       <c r="O53" s="42">
-        <f t="shared" si="28"/>
-        <v>1.778941555</v>
+        <f t="shared" si="32"/>
+        <v>0.3954301868</v>
       </c>
       <c r="P53" s="42">
-        <f t="shared" si="29"/>
-        <v>0.1765166222</v>
+        <f t="shared" si="32"/>
+        <v>0.2585189381</v>
       </c>
       <c r="Q53" s="42">
-        <f t="shared" si="30"/>
-        <v>0.2471512284</v>
+        <f t="shared" si="32"/>
+        <v>0.3165773097</v>
       </c>
       <c r="R53" s="3"/>
       <c r="S53" s="3">
-        <f t="shared" si="31"/>
-        <v>0.5656830415</v>
+        <f t="shared" si="29"/>
+        <v>0.2983839019</v>
       </c>
       <c r="T53" s="20">
-        <f t="shared" si="32"/>
-        <v>0.5656830415</v>
+        <f t="shared" si="30"/>
+        <v>0.2983839019</v>
       </c>
       <c r="U53" s="3"/>
     </row>
@@ -3016,19 +3029,19 @@
         <v>18</v>
       </c>
       <c r="B54" s="42">
-        <f t="shared" ref="B54:E54" si="34">POWER(B45*H45*O45,1/3)</f>
+        <f t="shared" ref="B54:E54" si="33">POWER(B45*H45*O45,1/3)</f>
         <v>0.2</v>
       </c>
       <c r="C54" s="42">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>0.3028534321</v>
       </c>
       <c r="D54" s="42">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>0.2320794417</v>
       </c>
       <c r="E54" s="42">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>1</v>
       </c>
       <c r="F54" s="36"/>
@@ -3046,29 +3059,29 @@
         <v>18</v>
       </c>
       <c r="N54" s="42">
-        <f t="shared" si="27"/>
-        <v>0.02752935202</v>
+        <f t="shared" ref="N54:Q54" si="34">B54/B$56</f>
+        <v>0.1021127106</v>
       </c>
       <c r="O54" s="42">
-        <f t="shared" si="28"/>
-        <v>0.1867771593</v>
+        <f t="shared" si="34"/>
+        <v>0.04151756801</v>
       </c>
       <c r="P54" s="42">
-        <f t="shared" si="29"/>
-        <v>0.04096587914</v>
+        <f t="shared" si="34"/>
+        <v>0.05999693082</v>
       </c>
       <c r="Q54" s="42">
-        <f t="shared" si="30"/>
-        <v>0.05735871911</v>
+        <f t="shared" si="34"/>
+        <v>0.07347108529</v>
       </c>
       <c r="R54" s="3"/>
       <c r="S54" s="3">
-        <f t="shared" si="31"/>
-        <v>0.0781577774</v>
+        <f t="shared" si="29"/>
+        <v>0.06927457368</v>
       </c>
       <c r="T54" s="20">
-        <f t="shared" si="32"/>
-        <v>0.0781577774</v>
+        <f t="shared" si="30"/>
+        <v>0.06927457368</v>
       </c>
       <c r="U54" s="3"/>
     </row>
@@ -3080,7 +3093,7 @@
         <v>12</v>
       </c>
       <c r="B56" s="14">
-        <f t="shared" ref="B56:E56" si="35">SUM(B51:B55)</f>
+        <f t="shared" ref="B56:E56" si="35">SUM(B51:B54)</f>
         <v>1.958620027</v>
       </c>
       <c r="C56" s="14">
@@ -3629,28 +3642,28 @@
         <v>15</v>
       </c>
       <c r="N70" s="42">
-        <f t="shared" ref="N70:N73" si="38">B70/$B$37</f>
-        <v>0.1376467601</v>
+        <f t="shared" ref="N70:Q70" si="37">B70/B$75</f>
+        <v>0.2417731183</v>
       </c>
       <c r="O70" s="42">
-        <f t="shared" ref="O70:O73" si="39">C70/$C$37</f>
-        <v>0.2693792778</v>
+        <f t="shared" si="37"/>
+        <v>0.2508058069</v>
       </c>
       <c r="P70" s="42">
-        <f t="shared" ref="P70:P73" si="40">D70/$D$37</f>
-        <v>0.5091620451</v>
+        <f t="shared" si="37"/>
+        <v>0.2197549394</v>
       </c>
       <c r="Q70" s="42">
-        <f t="shared" ref="Q70:Q73" si="41">E70/$E$37</f>
-        <v>0.1147174382</v>
+        <f t="shared" si="37"/>
+        <v>0.2072269305</v>
       </c>
       <c r="S70" s="3">
-        <f t="shared" ref="S70:S73" si="42">AVERAGE(N70:R70)</f>
-        <v>0.2577263803</v>
+        <f t="shared" ref="S70:S73" si="40">AVERAGE(N70:R70)</f>
+        <v>0.2298901988</v>
       </c>
       <c r="T70" s="20">
-        <f t="shared" ref="T70:T73" si="43">AVERAGE(N70:R70)</f>
-        <v>0.2577263803</v>
+        <f t="shared" ref="T70:T73" si="41">AVERAGE(N70:R70)</f>
+        <v>0.2298901988</v>
       </c>
       <c r="U70" s="3"/>
     </row>
@@ -3659,19 +3672,19 @@
         <v>16</v>
       </c>
       <c r="B71" s="42">
-        <f t="shared" ref="B71:E71" si="37">POWER(B62*H62*O62,1/3)</f>
+        <f t="shared" ref="B71:E71" si="38">POWER(B62*H62*O62,1/3)</f>
         <v>2.289428485</v>
       </c>
       <c r="C71" s="42">
-        <f t="shared" si="37"/>
+        <f t="shared" si="38"/>
         <v>1</v>
       </c>
       <c r="D71" s="42">
-        <f t="shared" si="37"/>
+        <f t="shared" si="38"/>
         <v>6.95205329</v>
       </c>
       <c r="E71" s="42">
-        <f t="shared" si="37"/>
+        <f t="shared" si="38"/>
         <v>6.214465012</v>
       </c>
       <c r="F71" s="36"/>
@@ -3689,28 +3702,28 @@
         <v>16</v>
       </c>
       <c r="N71" s="42">
-        <f t="shared" si="38"/>
-        <v>0.3151324135</v>
+        <f t="shared" ref="N71:Q71" si="39">B71/B$75</f>
+        <v>0.5535222639</v>
       </c>
       <c r="O71" s="42">
         <f t="shared" si="39"/>
-        <v>0.6167245918</v>
+        <v>0.5742019585</v>
       </c>
       <c r="P71" s="42">
+        <f t="shared" si="39"/>
+        <v>0.5296406672</v>
+      </c>
+      <c r="Q71" s="42">
+        <f t="shared" si="39"/>
+        <v>0.6439022546</v>
+      </c>
+      <c r="S71" s="3">
         <f t="shared" si="40"/>
-        <v>1.227152964</v>
-      </c>
-      <c r="Q71" s="42">
+        <v>0.5753167861</v>
+      </c>
+      <c r="T71" s="20">
         <f t="shared" si="41"/>
-        <v>0.356453753</v>
-      </c>
-      <c r="S71" s="3">
-        <f t="shared" si="42"/>
-        <v>0.6288659307</v>
-      </c>
-      <c r="T71" s="20">
-        <f t="shared" si="43"/>
-        <v>0.6288659307</v>
+        <v>0.5753167861</v>
       </c>
       <c r="U71" s="3"/>
     </row>
@@ -3719,19 +3732,19 @@
         <v>17</v>
       </c>
       <c r="B72" s="42">
-        <f t="shared" ref="B72:E72" si="44">POWER(B63*H63*O63,1/3)</f>
+        <f t="shared" ref="B72:E72" si="42">POWER(B63*H63*O63,1/3)</f>
         <v>0.3466806372</v>
       </c>
       <c r="C72" s="42">
-        <f t="shared" si="44"/>
+        <f t="shared" si="42"/>
         <v>0.1438423957</v>
       </c>
       <c r="D72" s="42">
-        <f t="shared" si="44"/>
+        <f t="shared" si="42"/>
         <v>1</v>
       </c>
       <c r="E72" s="42">
-        <f t="shared" si="44"/>
+        <f t="shared" si="42"/>
         <v>0.4367902324</v>
       </c>
       <c r="F72" s="36"/>
@@ -3749,28 +3762,28 @@
         <v>17</v>
       </c>
       <c r="N72" s="42">
-        <f t="shared" si="38"/>
-        <v>0.0477194665</v>
+        <f t="shared" ref="N72:Q72" si="43">B72/B$75</f>
+        <v>0.08381805869</v>
       </c>
       <c r="O72" s="42">
-        <f t="shared" si="39"/>
-        <v>0.08871114275</v>
+        <f t="shared" si="43"/>
+        <v>0.08259458531</v>
       </c>
       <c r="P72" s="42">
+        <f t="shared" si="43"/>
+        <v>0.07618478241</v>
+      </c>
+      <c r="Q72" s="42">
+        <f t="shared" si="43"/>
+        <v>0.04525734957</v>
+      </c>
+      <c r="S72" s="3">
         <f t="shared" si="40"/>
-        <v>0.1765166222</v>
-      </c>
-      <c r="Q72" s="42">
+        <v>0.071963694</v>
+      </c>
+      <c r="T72" s="20">
         <f t="shared" si="41"/>
-        <v>0.02505372825</v>
-      </c>
-      <c r="S72" s="3">
-        <f t="shared" si="42"/>
-        <v>0.08450023993</v>
-      </c>
-      <c r="T72" s="20">
-        <f t="shared" si="43"/>
-        <v>0.08450023993</v>
+        <v>0.071963694</v>
       </c>
       <c r="U72" s="3"/>
     </row>
@@ -3779,19 +3792,19 @@
         <v>18</v>
       </c>
       <c r="B73" s="42">
-        <f t="shared" ref="B73:E73" si="45">POWER(B64*H64*O64,1/3)</f>
+        <f t="shared" ref="B73:E73" si="44">POWER(B64*H64*O64,1/3)</f>
         <v>0.5</v>
       </c>
       <c r="C73" s="42">
-        <f t="shared" si="45"/>
+        <f t="shared" si="44"/>
         <v>0.1609148974</v>
       </c>
       <c r="D73" s="42">
-        <f t="shared" si="45"/>
+        <f t="shared" si="44"/>
         <v>2.289428485</v>
       </c>
       <c r="E73" s="42">
-        <f t="shared" si="45"/>
+        <f t="shared" si="44"/>
         <v>1</v>
       </c>
       <c r="F73" s="36"/>
@@ -3809,28 +3822,28 @@
         <v>18</v>
       </c>
       <c r="N73" s="42">
-        <f t="shared" si="38"/>
-        <v>0.06882338006</v>
+        <f t="shared" ref="N73:Q73" si="45">B73/B$75</f>
+        <v>0.1208865591</v>
       </c>
       <c r="O73" s="42">
-        <f t="shared" si="39"/>
-        <v>0.09924017444</v>
+        <f t="shared" si="45"/>
+        <v>0.09239764926</v>
       </c>
       <c r="P73" s="42">
+        <f t="shared" si="45"/>
+        <v>0.174419611</v>
+      </c>
+      <c r="Q73" s="42">
+        <f t="shared" si="45"/>
+        <v>0.1036134653</v>
+      </c>
+      <c r="S73" s="3">
         <f t="shared" si="40"/>
-        <v>0.404122183</v>
-      </c>
-      <c r="Q73" s="42">
+        <v>0.1228293212</v>
+      </c>
+      <c r="T73" s="20">
         <f t="shared" si="41"/>
-        <v>0.05735871911</v>
-      </c>
-      <c r="S73" s="3">
-        <f t="shared" si="42"/>
-        <v>0.1573861142</v>
-      </c>
-      <c r="T73" s="20">
-        <f t="shared" si="43"/>
-        <v>0.1573861142</v>
+        <v>0.1228293212</v>
       </c>
       <c r="U73" s="3"/>
     </row>
@@ -4390,29 +4403,29 @@
         <v>15</v>
       </c>
       <c r="N89" s="42">
-        <f t="shared" ref="N89:N92" si="50">B89/$B$37</f>
-        <v>0.1376467601</v>
+        <f t="shared" ref="N89:Q89" si="49">B89/B$94</f>
+        <v>0.5165469148</v>
       </c>
       <c r="O89" s="42">
-        <f t="shared" ref="O89:O92" si="51">C89/$C$37</f>
-        <v>1.411946848</v>
+        <f t="shared" si="49"/>
+        <v>0.5738738001</v>
       </c>
       <c r="P89" s="42">
-        <f t="shared" ref="P89:P92" si="52">D89/$D$37</f>
-        <v>0.6609552291</v>
+        <f t="shared" si="49"/>
+        <v>0.3066533497</v>
       </c>
       <c r="Q89" s="42">
-        <f t="shared" ref="Q89:Q92" si="53">E89/$E$37</f>
-        <v>0.2471512284</v>
+        <f t="shared" si="49"/>
+        <v>0.5585525225</v>
       </c>
       <c r="R89" s="36"/>
       <c r="S89" s="3">
-        <f t="shared" ref="S89:S92" si="54">AVERAGE(N89:R89)</f>
-        <v>0.6144250164</v>
+        <f t="shared" ref="S89:S92" si="52">AVERAGE(N89:R89)</f>
+        <v>0.4889066468</v>
       </c>
       <c r="T89" s="20">
-        <f t="shared" ref="T89:T92" si="55">AVERAGE(N89:R89)</f>
-        <v>0.6144250164</v>
+        <f t="shared" ref="T89:T92" si="53">AVERAGE(N89:R89)</f>
+        <v>0.4889066468</v>
       </c>
       <c r="U89" s="3"/>
     </row>
@@ -4421,19 +4434,19 @@
         <v>16</v>
       </c>
       <c r="B90" s="42">
-        <f t="shared" ref="B90:E90" si="49">POWER(B81*H81*O81,1/3)</f>
+        <f t="shared" ref="B90:E90" si="50">POWER(B81*H81*O81,1/3)</f>
         <v>0.4367902324</v>
       </c>
       <c r="C90" s="42">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>1</v>
       </c>
       <c r="D90" s="42">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>5</v>
       </c>
       <c r="E90" s="42">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>2</v>
       </c>
       <c r="F90" s="36"/>
@@ -4451,29 +4464,29 @@
         <v>16</v>
       </c>
       <c r="N90" s="42">
-        <f t="shared" si="50"/>
-        <v>0.06012276034</v>
+        <f t="shared" ref="N90:Q90" si="51">B90/B$94</f>
+        <v>0.225622647</v>
       </c>
       <c r="O90" s="42">
         <f t="shared" si="51"/>
-        <v>0.6167245918</v>
+        <v>0.2506624705</v>
       </c>
       <c r="P90" s="42">
-        <f t="shared" si="52"/>
-        <v>0.8825831112</v>
+        <f t="shared" si="51"/>
+        <v>0.409478669</v>
       </c>
       <c r="Q90" s="42">
-        <f t="shared" si="53"/>
-        <v>0.1147174382</v>
+        <f t="shared" si="51"/>
+        <v>0.2592571151</v>
       </c>
       <c r="R90" s="36"/>
       <c r="S90" s="3">
-        <f t="shared" si="54"/>
-        <v>0.4185369754</v>
+        <f t="shared" si="52"/>
+        <v>0.2862552254</v>
       </c>
       <c r="T90" s="20">
-        <f t="shared" si="55"/>
-        <v>0.4185369754</v>
+        <f t="shared" si="53"/>
+        <v>0.2862552254</v>
       </c>
       <c r="U90" s="3"/>
     </row>
@@ -4482,19 +4495,19 @@
         <v>17</v>
       </c>
       <c r="B91" s="42">
-        <f t="shared" ref="B91:E91" si="56">POWER(B82*H82*O82,1/3)</f>
+        <f t="shared" ref="B91:E91" si="54">POWER(B82*H82*O82,1/3)</f>
         <v>0.267062903</v>
       </c>
       <c r="C91" s="42">
-        <f t="shared" si="56"/>
+        <f t="shared" si="54"/>
         <v>0.2</v>
       </c>
       <c r="D91" s="42">
-        <f t="shared" si="56"/>
+        <f t="shared" si="54"/>
         <v>1</v>
       </c>
       <c r="E91" s="42">
-        <f t="shared" si="56"/>
+        <f t="shared" si="54"/>
         <v>0.405480133</v>
       </c>
       <c r="F91" s="36"/>
@@ -4512,29 +4525,29 @@
         <v>17</v>
       </c>
       <c r="N91" s="42">
-        <f t="shared" si="50"/>
-        <v>0.03676034335</v>
+        <f t="shared" ref="N91:Q91" si="55">B91/B$94</f>
+        <v>0.1379505186</v>
       </c>
       <c r="O91" s="42">
-        <f t="shared" si="51"/>
-        <v>0.1233449184</v>
+        <f t="shared" si="55"/>
+        <v>0.0501324941</v>
       </c>
       <c r="P91" s="42">
-        <f t="shared" si="52"/>
-        <v>0.1765166222</v>
+        <f t="shared" si="55"/>
+        <v>0.08189573379</v>
       </c>
       <c r="Q91" s="42">
-        <f t="shared" si="53"/>
-        <v>0.02325782106</v>
+        <f t="shared" si="55"/>
+        <v>0.05256180477</v>
       </c>
       <c r="R91" s="36"/>
       <c r="S91" s="3">
-        <f t="shared" si="54"/>
-        <v>0.08996992625</v>
+        <f t="shared" si="52"/>
+        <v>0.08063513782</v>
       </c>
       <c r="T91" s="20">
-        <f t="shared" si="55"/>
-        <v>0.08996992625</v>
+        <f t="shared" si="53"/>
+        <v>0.08063513782</v>
       </c>
       <c r="U91" s="3"/>
     </row>
@@ -4543,19 +4556,19 @@
         <v>18</v>
       </c>
       <c r="B92" s="42">
-        <f t="shared" ref="B92:E92" si="57">POWER(B83*H83*O83,1/3)</f>
+        <f t="shared" ref="B92:E92" si="56">POWER(B83*H83*O83,1/3)</f>
         <v>0.2320794417</v>
       </c>
       <c r="C92" s="42">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>0.5</v>
       </c>
       <c r="D92" s="42">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>2.466212074</v>
       </c>
       <c r="E92" s="42">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>1</v>
       </c>
       <c r="F92" s="36"/>
@@ -4573,29 +4586,29 @@
         <v>18</v>
       </c>
       <c r="N92" s="42">
-        <f t="shared" si="50"/>
-        <v>0.03194498324</v>
+        <f t="shared" ref="N92:Q92" si="57">B92/B$94</f>
+        <v>0.1198799196</v>
       </c>
       <c r="O92" s="42">
-        <f t="shared" si="51"/>
-        <v>0.3083622959</v>
+        <f t="shared" si="57"/>
+        <v>0.1253312353</v>
       </c>
       <c r="P92" s="42">
-        <f t="shared" si="52"/>
-        <v>0.4353274251</v>
+        <f t="shared" si="57"/>
+        <v>0.2019722475</v>
       </c>
       <c r="Q92" s="42">
-        <f t="shared" si="53"/>
-        <v>0.05735871911</v>
+        <f t="shared" si="57"/>
+        <v>0.1296285576</v>
       </c>
       <c r="R92" s="36"/>
       <c r="S92" s="3">
-        <f t="shared" si="54"/>
-        <v>0.2082483558</v>
+        <f t="shared" si="52"/>
+        <v>0.14420299</v>
       </c>
       <c r="T92" s="20">
-        <f t="shared" si="55"/>
-        <v>0.2082483558</v>
+        <f t="shared" si="53"/>
+        <v>0.14420299</v>
       </c>
       <c r="U92" s="3"/>
     </row>
@@ -4753,24 +4766,24 @@
       <c r="A99" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="B99" s="34">
+      <c r="B99" s="51">
         <f t="shared" ref="B99:B102" si="59">S32</f>
         <v>0.1456032916</v>
       </c>
       <c r="C99" s="34">
         <f t="shared" ref="C99:C102" si="60">S51</f>
-        <v>0.6862173094</v>
+        <v>0.4739359641</v>
       </c>
       <c r="D99" s="34">
         <f t="shared" ref="D99:D102" si="61">S70</f>
-        <v>0.2577263803</v>
+        <v>0.2298901988</v>
       </c>
       <c r="E99" s="34">
         <f t="shared" ref="E99:E102" si="62">S89</f>
-        <v>0.6144250164</v>
+        <v>0.4889066468</v>
       </c>
       <c r="F99" s="3"/>
-      <c r="G99" s="51" t="s">
+      <c r="G99" s="52" t="s">
         <v>5</v>
       </c>
       <c r="H99" s="34">
@@ -4795,24 +4808,24 @@
       <c r="A100" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B100" s="34">
+      <c r="B100" s="51">
         <f t="shared" si="59"/>
         <v>0.5842161629</v>
       </c>
       <c r="C100" s="34">
         <f t="shared" si="60"/>
-        <v>0.2279031583</v>
+        <v>0.1584055603</v>
       </c>
       <c r="D100" s="34">
         <f t="shared" si="61"/>
-        <v>0.6288659307</v>
+        <v>0.5753167861</v>
       </c>
       <c r="E100" s="34">
         <f t="shared" si="62"/>
-        <v>0.4185369754</v>
+        <v>0.2862552254</v>
       </c>
       <c r="F100" s="3"/>
-      <c r="G100" s="51" t="s">
+      <c r="G100" s="52" t="s">
         <v>6</v>
       </c>
       <c r="H100" s="34">
@@ -4837,24 +4850,24 @@
       <c r="A101" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="B101" s="34">
+      <c r="B101" s="53">
         <f t="shared" si="59"/>
         <v>0.2177412344</v>
       </c>
       <c r="C101" s="34">
         <f t="shared" si="60"/>
-        <v>0.5656830415</v>
+        <v>0.2983839019</v>
       </c>
       <c r="D101" s="34">
         <f t="shared" si="61"/>
-        <v>0.08450023993</v>
+        <v>0.071963694</v>
       </c>
       <c r="E101" s="34">
         <f t="shared" si="62"/>
-        <v>0.08996992625</v>
+        <v>0.08063513782</v>
       </c>
       <c r="F101" s="3"/>
-      <c r="G101" s="51" t="s">
+      <c r="G101" s="52" t="s">
         <v>7</v>
       </c>
       <c r="H101" s="34">
@@ -4879,24 +4892,24 @@
       <c r="A102" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="B102" s="34">
+      <c r="B102" s="51">
         <f t="shared" si="59"/>
         <v>0.05243931108</v>
       </c>
       <c r="C102" s="34">
         <f t="shared" si="60"/>
-        <v>0.0781577774</v>
+        <v>0.06927457368</v>
       </c>
       <c r="D102" s="34">
         <f t="shared" si="61"/>
-        <v>0.1573861142</v>
+        <v>0.1228293212</v>
       </c>
       <c r="E102" s="34">
         <f t="shared" si="62"/>
-        <v>0.2082483558</v>
+        <v>0.14420299</v>
       </c>
       <c r="F102" s="3"/>
-      <c r="G102" s="51" t="s">
+      <c r="G102" s="52" t="s">
         <v>8</v>
       </c>
       <c r="H102" s="34">
@@ -4919,10 +4932,22 @@
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="3"/>
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="D103" s="3"/>
-      <c r="E103" s="3"/>
+      <c r="B103" s="54">
+        <f t="shared" ref="B103:E103" si="64">SUM(B99:B102)</f>
+        <v>1</v>
+      </c>
+      <c r="C103" s="3">
+        <f t="shared" si="64"/>
+        <v>1</v>
+      </c>
+      <c r="D103" s="3">
+        <f t="shared" si="64"/>
+        <v>1</v>
+      </c>
+      <c r="E103" s="3">
+        <f t="shared" si="64"/>
+        <v>1</v>
+      </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
@@ -4964,13 +4989,13 @@
       <c r="U104" s="3"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="52" t="s">
+      <c r="A105" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="B105" s="53" t="s">
+      <c r="B105" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C105" s="53" t="s">
+      <c r="C105" s="56" t="s">
         <v>11</v>
       </c>
       <c r="D105" s="3"/>
@@ -4993,16 +5018,16 @@
       <c r="U105" s="3"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="54" t="s">
+      <c r="A106" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="B106" s="55">
+      <c r="B106" s="58">
         <f t="array" ref="B106:B109">MMULT(B99:E102,H99:H102)</f>
-        <v>0.3145077404</v>
-      </c>
-      <c r="C106" s="56">
-        <f t="shared" ref="C106:C109" si="64">B106</f>
-        <v>0.3145077404</v>
+        <v>0.265567218</v>
+      </c>
+      <c r="C106" s="59">
+        <f t="shared" ref="C106:C109" si="65">B106</f>
+        <v>0.265567218</v>
       </c>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
@@ -5024,15 +5049,15 @@
       <c r="U106" s="3"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="57" t="s">
+      <c r="A107" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="B107" s="58">
-        <v>0.5257602969559335</v>
-      </c>
-      <c r="C107" s="59">
-        <f t="shared" si="64"/>
-        <v>0.525760297</v>
+      <c r="B107" s="61">
+        <v>0.4801578157541191</v>
+      </c>
+      <c r="C107" s="62">
+        <f t="shared" si="65"/>
+        <v>0.4801578158</v>
       </c>
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
@@ -5054,15 +5079,15 @@
       <c r="U107" s="3"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="60" t="s">
+      <c r="A108" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="B108" s="61">
-        <v>0.187634044604344</v>
-      </c>
-      <c r="C108" s="62">
-        <f t="shared" si="64"/>
-        <v>0.1876340446</v>
+      <c r="B108" s="64">
+        <v>0.1677091942462168</v>
+      </c>
+      <c r="C108" s="65">
+        <f t="shared" si="65"/>
+        <v>0.1677091942</v>
       </c>
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
@@ -5088,11 +5113,11 @@
         <v>18</v>
       </c>
       <c r="B109" s="34">
-        <v>0.10830608238168707</v>
+        <v>0.0865657719796254</v>
       </c>
       <c r="C109" s="33">
-        <f t="shared" si="64"/>
-        <v>0.1083060824</v>
+        <f t="shared" si="65"/>
+        <v>0.08656577198</v>
       </c>
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
@@ -10444,14 +10469,14 @@
     <row r="1" ht="15.75" customHeight="1"/>
     <row r="2" ht="15.75" customHeight="1"/>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="63" t="s">
+      <c r="C3" s="67"/>
+      <c r="D3" s="66" t="s">
         <v>35</v>
       </c>
     </row>
@@ -10462,7 +10487,7 @@
       <c r="B4" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="64"/>
+      <c r="C4" s="67"/>
       <c r="D4" s="34" t="s">
         <v>41</v>
       </c>
@@ -10474,7 +10499,7 @@
       <c r="B5" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="64"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="34" t="s">
         <v>6</v>
       </c>
@@ -10486,8 +10511,8 @@
       <c r="B6" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="64"/>
-      <c r="D6" s="51" t="s">
+      <c r="C6" s="67"/>
+      <c r="D6" s="52" t="s">
         <v>7</v>
       </c>
     </row>
@@ -10498,8 +10523,8 @@
       <c r="B7" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="64"/>
-      <c r="D7" s="51" t="s">
+      <c r="C7" s="67"/>
+      <c r="D7" s="52" t="s">
         <v>8</v>
       </c>
     </row>
@@ -10510,22 +10535,22 @@
       <c r="B8" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="64"/>
+      <c r="C8" s="67"/>
       <c r="D8" s="34" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="64"/>
-      <c r="B9" s="64"/>
-      <c r="C9" s="64"/>
-      <c r="D9" s="64"/>
+      <c r="A9" s="67"/>
+      <c r="B9" s="67"/>
+      <c r="C9" s="67"/>
+      <c r="D9" s="67"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="64"/>
-      <c r="B10" s="64"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
+      <c r="A10" s="67"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
     </row>
     <row r="11" ht="15.75" customHeight="1"/>
     <row r="12" ht="15.75" customHeight="1"/>

</xml_diff>